<commit_message>
Update HS summary notes: R290 not F-gas, drop advance-payment remark, keep BL totals
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ULe8MDenbzgA59JAYzcvjt
</commit_message>
<xml_diff>
--- a/output/HS_sumar_KLI20260422002_MRSU9864772.xlsx
+++ b/output/HS_sumar_KLI20260422002_MRSU9864772.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -669,53 +669,37 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>1) Fakturační mezisoučet položek = 954 899,60 CNY. Na faktuře je odečtena záloha „PAYMENT BY TT IN ADVANCE“ -190 979,92 CNY, takže „TOTAL AMOUNT“ = 763 919,68 CNY je pouze doplatek. Do celní hodnoty patří celková cena zboží 954 899,60 CNY (záloha je součástí ceny placené za zboží).</t>
+          <t>1) Dodací podmínka FOB BEIJIAO (Freight Collect): k ceně zboží je nutné připočíst námořní přepravné a případné pojištění do místa vstupu do EU (Bremerhaven). Doklad o dopravě bude zaslán spolu s MRN.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>2) Chladivo všech jednotek je R290 (propan) – uhlovodík, NENÍ to částečně fluorovaný uhlovodík (HFC). TARIC koncovka 91 („Předem naplněná částečně fluorovanými uhlovodíky (HFC)“) se proto nepoužije → navrženo 8418 61 00 99. Dle konverzace čeká na potvrzení (Věrka).</t>
+          <t>2) Chladivo všech jednotek je R290 (propan) – doloženo výrobními štítky, technickými listy i Přílohou č. 1. R290 není fluorovaný skleníkový plyn (není uveden v příloze I nařízení (EU) 2024/573) → zboží NENÍ předem naplněné HFC, TARIC koncovka 91 se nepoužije → deklarovat 8418 61 00 99. Bez F-gas povinností (kvóty, F-gas portál).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>3) FOB BEIJIAO: k ceně zboží je nutné připočíst námořní přepravné a případné pojištění do místa vstupu do EU (Bremerhaven) – doklad o dopravě přijde s MRN.</t>
+          <t>3) Platební podmínka: TT + OA 30 dní od data B/L.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>4) Nesrovnalost: Příloha č. 1 k Vyhlášení o shodě uvádí v řádku TOTAL 69 ks, správně má být 60 ks (součet položek i faktura/PL = 60).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>5) Návrh CO v sešitu CIPL uvádí HS 8415 – správně má být 8418 61. Zkontrolovat finální originál CO.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
-        <is>
-          <t>6) Platební podmínka: TT + OA 30 dní od data B/L.</t>
+          <t>4) Návrh CO v sešitu CIPL uvádí HS 8415 – správně má být 8418 61. Zkontrolovat finální originál Certificate of Origin.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="5">
     <mergeCell ref="A15:I15"/>
     <mergeCell ref="A19:I19"/>
     <mergeCell ref="A17:I17"/>
     <mergeCell ref="A18:I18"/>
-    <mergeCell ref="A20:I20"/>
-    <mergeCell ref="A21:I21"/>
     <mergeCell ref="A16:I16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>